<commit_message>
feat:  removed latest Imported Date related logic
</commit_message>
<xml_diff>
--- a/src/Apha.FPSApps/Apha.FPSApps.Web/wwwroot/templates/PACT/InvoiceImport-Template.xlsx
+++ b/src/Apha.FPSApps/Apha.FPSApps.Web/wwwroot/templates/PACT/InvoiceImport-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vinay-Work\Pact\Working\src\Apha.FPSApps\Apha.FPSApps.Web\wwwroot\templates\PACT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73595314-7EAE-4739-8889-0C1EA6DCEF29}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8015E99E-881D-4FBE-A175-152C8A31087D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18900" windowHeight="5130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>Project Parent</t>
   </si>
@@ -41,9 +41,6 @@
   </si>
   <si>
     <t>Type</t>
-  </si>
-  <si>
-    <t>Id</t>
   </si>
   <si>
     <t>Profit Loss</t>
@@ -413,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -424,10 +421,9 @@
     <col min="6" max="6" width="10.5703125" style="1" customWidth="1"/>
     <col min="7" max="7" width="5.85546875" customWidth="1"/>
     <col min="8" max="8" width="5.140625" customWidth="1"/>
-    <col min="9" max="9" width="2.7109375" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -444,16 +440,13 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>5</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Removed Type property
</commit_message>
<xml_diff>
--- a/src/Apha.FPSApps/Apha.FPSApps.Web/wwwroot/templates/PACT/InvoiceImport-Template.xlsx
+++ b/src/Apha.FPSApps/Apha.FPSApps.Web/wwwroot/templates/PACT/InvoiceImport-Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Vinay-Work\Pact\Working\src\Apha.FPSApps\Apha.FPSApps.Web\wwwroot\templates\PACT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8015E99E-881D-4FBE-A175-152C8A31087D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBDAA40-8562-4F54-A2C4-11621E5DD8F1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="18900" windowHeight="5130" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Project Parent</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>Detail</t>
-  </si>
-  <si>
-    <t>Type</t>
   </si>
   <si>
     <t>Profit Loss</t>
@@ -410,7 +407,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -418,12 +415,11 @@
     <col min="3" max="3" width="8.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.5703125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="5.85546875" customWidth="1"/>
-    <col min="8" max="8" width="5.140625" customWidth="1"/>
+    <col min="6" max="6" width="10.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -440,13 +436,10 @@
         <v>4</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>5</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>